<commit_message>
n8n board refresh 2026-07-12T17:38:31Z
</commit_message>
<xml_diff>
--- a/app/reports/CPOP_research.xlsx
+++ b/app/reports/CPOP_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-11 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-12 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -1524,10 +1524,10 @@
       </c>
       <c r="D5" s="32" t="n"/>
       <c r="E5" s="32" t="n">
-        <v>-25.5</v>
+        <v>-212.38</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>0.04</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="6">

</xml_diff>